<commit_message>
FC BoM fixes: R40 LCSC number, LPS22HH barometer, MCU sourcing note
- R40 47k 0402: C25819 (0603) -> C25792 (0402WGF4702TCE)
- U4: LPS22HBTR (out of stock) -> LPS22HHTR C2827824, same HLGA-10 footprint and pinout
- U2 STM32WB55CGU6 out of stock at LCSC/JLC: consigned part / Global Sourcing note

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0189Xg6tRAL4bRZ656VQBtPX
</commit_message>
<xml_diff>
--- a/00 - Docs/00 - FC_Docs/ACwing_FC_A_BoM.xlsx
+++ b/00 - Docs/00 - FC_Docs/ACwing_FC_A_BoM.xlsx
@@ -761,7 +761,7 @@
     <t xml:space="preserve">0402WGF4702TCE</t>
   </si>
   <si>
-    <t xml:space="preserve">C25819</t>
+    <t xml:space="preserve">C25792</t>
   </si>
   <si>
     <t xml:space="preserve">Resistor, 47 kOhm, 1%, 1/16 W</t>
@@ -881,7 +881,7 @@
     <t xml:space="preserve">MCU, Cortex-M4 + M0+ radio core, BLE 5 / 802.15.4, 1 MB flash, 256 KB RAM, SMPS</t>
   </si>
   <si>
-    <t xml:space="preserve">EP to GND through a 3x3 via array</t>
+    <t xml:space="preserve">EP to GND through a 3x3 via array. Out of stock at LCSC/JLC (2026-10-27): consigned part (buy at Mouser/DigiKey/ST and ship to JLC) or JLC Global Sourcing</t>
   </si>
   <si>
     <t xml:space="preserve">U3</t>
@@ -908,22 +908,22 @@
     <t xml:space="preserve">U4</t>
   </si>
   <si>
-    <t xml:space="preserve">LPS22HB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LPS22HBTR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C94049</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HLGA-10, 2 x 2 x 0.76 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pressure sensor (barometer), 260-1260 hPa, I2C/SPI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Altitude hold; address 0x5D. Keep the vent hole clear. Out of stock at LCSC/JLC on 2026-10-16: use JLC Global Sourcing or send your own parts (consigned)</t>
+    <t xml:space="preserve">LPS22HH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LPS22HHTR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2827824</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HLGA-10, 2 x 2 x 0.73 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pressure sensor (barometer), 260-1260 hPa, I2C/SPI, 24-bit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Altitude hold; address 0x5D (WHO_AM_I 0xB3). Keep the vent hole clear. Replaces LPS22HBTR (out of stock): same HLGA-10 2 x 2 footprint and pinout; low LCSC stock on 2026-10-27, check before ordering</t>
   </si>
   <si>
     <t xml:space="preserve">U5</t>
@@ -1346,7 +1346,7 @@
     <t xml:space="preserve">LCSC C25105 (JLC Basic)</t>
   </si>
   <si>
-    <t xml:space="preserve">LCSC C25819 (JLC Basic)</t>
+    <t xml:space="preserve">LCSC C25792 (JLC Basic)</t>
   </si>
   <si>
     <t xml:space="preserve">LCSC C25756 (JLC Basic)</t>
@@ -1367,16 +1367,16 @@
     <t xml:space="preserve">LCSC C404023</t>
   </si>
   <si>
-    <t xml:space="preserve">Mouser/DigiKey: 7.22 USD @10, 6.16-6.31 USD @100</t>
+    <t xml:space="preserve">Out of stock at LCSC/JLC (2026-10-27): consigned part; Mouser/DigiKey 7.22 USD @10, 6.16-6.31 USD @100</t>
   </si>
   <si>
     <t xml:space="preserve">LCSC C2655002</t>
   </si>
   <si>
-    <t xml:space="preserve">LCSC C94049</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Out of stock at LCSC: reference price; buy where you found stock</t>
+    <t xml:space="preserve">LCSC C2827824</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaces LPS22HBTR (out of stock); 70 pcs at LCSC on 2026-10-27</t>
   </si>
   <si>
     <t xml:space="preserve">LCSC C2798213</t>
@@ -3684,7 +3684,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="n">
         <v>46</v>
       </c>
@@ -3754,7 +3754,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="n">
         <v>48</v>
       </c>
@@ -5824,7 +5824,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="n">
         <v>39</v>
       </c>
@@ -5915,18 +5915,18 @@
         <v>449</v>
       </c>
       <c r="F46" s="15" t="n">
-        <v>2.6466</v>
+        <v>3.9895</v>
       </c>
       <c r="G46" s="16" t="n">
         <f aca="false">C46*F46</f>
-        <v>2.6466</v>
+        <v>3.9895</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>2.0382</v>
+        <v>3.9895</v>
       </c>
       <c r="I46" s="16" t="n">
         <f aca="false">C46*H46</f>
-        <v>2.0382</v>
+        <v>3.9895</v>
       </c>
       <c r="J46" s="8" t="s">
         <v>391</v>
@@ -6223,12 +6223,12 @@
       <c r="F55" s="19"/>
       <c r="G55" s="22" t="n">
         <f aca="false">SUM(G6:G53)</f>
-        <v>28.1607</v>
+        <v>29.5036</v>
       </c>
       <c r="H55" s="19"/>
       <c r="I55" s="22" t="n">
         <f aca="false">SUM(I6:I53)</f>
-        <v>22.6596</v>
+        <v>24.6109</v>
       </c>
       <c r="J55" s="19"/>
       <c r="K55" s="19" t="s">
@@ -6246,12 +6246,12 @@
       <c r="F56" s="19"/>
       <c r="G56" s="23" t="n">
         <f aca="false">G55*C3</f>
-        <v>25.907844</v>
+        <v>27.143312</v>
       </c>
       <c r="H56" s="19"/>
       <c r="I56" s="23" t="n">
         <f aca="false">I55*C3</f>
-        <v>20.846832</v>
+        <v>22.642028</v>
       </c>
       <c r="J56" s="19"/>
       <c r="K56" s="19" t="s">
@@ -6269,12 +6269,12 @@
       <c r="F57" s="19"/>
       <c r="G57" s="23" t="n">
         <f aca="false">G55*10</f>
-        <v>281.607</v>
+        <v>295.036</v>
       </c>
       <c r="H57" s="19"/>
       <c r="I57" s="23" t="n">
         <f aca="false">I55*100</f>
-        <v>2265.96</v>
+        <v>2461.09</v>
       </c>
       <c r="J57" s="19"/>
       <c r="K57" s="19" t="s">
@@ -6292,12 +6292,12 @@
       <c r="F58" s="19"/>
       <c r="G58" s="24" t="n">
         <f aca="false">(G44+G43+G45+G46)/G55</f>
-        <v>0.608962135174197</v>
+        <v>0.626760802071612</v>
       </c>
       <c r="H58" s="19"/>
       <c r="I58" s="24" t="n">
         <f aca="false">(I44+I43+I45+I46)/I55</f>
-        <v>0.589079242352027</v>
+        <v>0.621659508591722</v>
       </c>
       <c r="J58" s="19"/>
       <c r="K58" s="19" t="s">

</xml_diff>

<commit_message>
FC: XL-2020RGBC-WS2812B LEDs, D11 Schottky replaced by 0R link R49
- D1-D4: XINGLIGHT XL-2020RGBC-WS2812B (C5349955), same footprint and pinout (WS2812B-2020 out of stock)
- D11 RB521S30 -> R49 0R 0402 at the same place: VLED = VSYS, LEDs above their 3.5 V minimum on 1S
- BoM, JLC BoM, CPL, schematic PDF, Gerber, STEP, PCB view regenerated; DRC 0

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0189Xg6tRAL4bRZ656VQBtPX
</commit_message>
<xml_diff>
--- a/00 - Docs/00 - FC_Docs/ACwing_FC_A_BoM.xlsx
+++ b/00 - Docs/00 - FC_Docs/ACwing_FC_A_BoM.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="833" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="465">
   <si>
     <t xml:space="preserve">ACwing FC rev A - assembly BoM (1 board)</t>
   </si>
@@ -332,22 +332,22 @@
     <t xml:space="preserve">D1, D2, D3, D4</t>
   </si>
   <si>
-    <t xml:space="preserve">WS2812B-2020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Worldsemi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C965555</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.0 x 2.0 x 0.84 mm, 4 pad</t>
+    <t xml:space="preserve">XL-2020RGBC-WS2812B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XINGLIGHT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5349955</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.0 x 2.0 x 0.65 mm, 4 pad (WS2812B-2020 footprint and pinout)</t>
   </si>
   <si>
     <t xml:space="preserve">LED, RGB addressable, integrated driver, 2.0 x 2.0 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">Status LEDs D1 rear, D2 left, D3 front, D4 right: one chain from PA7 (TIM17_CH1 + DMA); D3 / D4 supply pins face away from the magnetometer</t>
+    <t xml:space="preserve">Status LEDs D1 rear, D2 left, D3 front, D4 right: one chain from PA7 (TIM17_CH1 + DMA); D3 / D4 supply pins face away from the magnetometer. VDD 3.5-5.5 V (replaces WS2812B-2020, out of stock)</t>
   </si>
   <si>
     <t xml:space="preserve">D9</t>
@@ -374,30 +374,6 @@
     <t xml:space="preserve">USB VBUS -&gt; VSYS</t>
   </si>
   <si>
-    <t xml:space="preserve">D11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RB521S30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RB521S30T1G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">onsemi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C8523</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOD-523</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diode, Schottky, 30 V, 200 mA, SOD-523</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VSYS -&gt; VLED (keeps the LEDs below their VDD max with USB 5 V)</t>
-  </si>
-  <si>
     <t xml:space="preserve">J1</t>
   </si>
   <si>
@@ -731,7 +707,7 @@
     <t xml:space="preserve">Resistor, 0 Ohm jumper, 1/16 W</t>
   </si>
   <si>
-    <t xml:space="preserve">Antenna tuning, series position (replace with L/C after tuning). JLC Basic part</t>
+    <t xml:space="preserve">R34: antenna tuning, series position (replace with L/C after tuning); R49: VSYS -&gt; VLED link (replaces the Schottky). JLC Basic part</t>
   </si>
   <si>
     <t xml:space="preserve">R39</t>
@@ -842,6 +818,9 @@
     <t xml:space="preserve">Buck feedback, bottom. JLC Basic part</t>
   </si>
   <si>
+    <t xml:space="preserve">R49</t>
+  </si>
+  <si>
     <t xml:space="preserve">U1</t>
   </si>
   <si>
@@ -1262,18 +1241,15 @@
     <t xml:space="preserve">10 nF 50 V X7R</t>
   </si>
   <si>
-    <t xml:space="preserve">LCSC C965555</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Worldsemi RGB LED, price estimated</t>
+    <t xml:space="preserve">LCSC C5349955</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XINGLIGHT, ~94k in stock on 2026-10-27 (replaces WS2812B-2020)</t>
   </si>
   <si>
     <t xml:space="preserve">LCSC C110921</t>
   </si>
   <si>
-    <t xml:space="preserve">LCSC C8523</t>
-  </si>
-  <si>
     <t xml:space="preserve">LCSC C165948</t>
   </si>
   <si>
@@ -1338,6 +1314,9 @@
   </si>
   <si>
     <t xml:space="preserve">LCSC C25076 (JLC Basic)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R34, R49</t>
   </si>
   <si>
     <t xml:space="preserve">LCSC C17168 (JLC Basic)</t>
@@ -2634,7 +2613,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="n">
         <v>16</v>
       </c>
@@ -2733,7 +2712,7 @@
         <v>122</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="K22" s="8" t="s">
         <v>123</v>
@@ -2779,7 +2758,7 @@
         <v>20</v>
       </c>
       <c r="B24" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>132</v>
@@ -2791,22 +2770,22 @@
         <v>134</v>
       </c>
       <c r="F24" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G24" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="G24" s="8" t="s">
+      <c r="H24" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="H24" s="8" t="s">
+      <c r="I24" s="8" t="s">
         <v>137</v>
-      </c>
-      <c r="I24" s="8" t="s">
-        <v>138</v>
       </c>
       <c r="J24" s="8" t="s">
         <v>19</v>
       </c>
       <c r="K24" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2814,34 +2793,34 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C25" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="D25" s="6" t="s">
-        <v>141</v>
-      </c>
       <c r="E25" s="6" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="F25" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="G25" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="G25" s="6" t="s">
-        <v>143</v>
-      </c>
       <c r="H25" s="6" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="J25" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2852,34 +2831,34 @@
         <v>1</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="J26" s="8" t="s">
         <v>19</v>
       </c>
       <c r="K26" s="8" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="n">
         <v>23</v>
       </c>
@@ -2887,34 +2866,34 @@
         <v>1</v>
       </c>
       <c r="C27" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="H27" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="I27" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="E27" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="G27" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="H27" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="I27" s="6" t="s">
-        <v>138</v>
-      </c>
       <c r="J27" s="6" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="K27" s="6" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="n">
         <v>24</v>
       </c>
@@ -2937,16 +2916,16 @@
         <v>157</v>
       </c>
       <c r="H28" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="I28" s="8" t="s">
         <v>158</v>
-      </c>
-      <c r="I28" s="8" t="s">
-        <v>159</v>
       </c>
       <c r="J28" s="8" t="s">
         <v>28</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2957,31 +2936,31 @@
         <v>1</v>
       </c>
       <c r="C29" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="D29" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="E29" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="F29" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="G29" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="H29" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="G29" s="6" t="s">
+      <c r="I29" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="H29" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="I29" s="6" t="s">
+      <c r="J29" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K29" s="6" t="s">
         <v>166</v>
-      </c>
-      <c r="J29" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="K29" s="6" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2992,31 +2971,31 @@
         <v>1</v>
       </c>
       <c r="C30" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="D30" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="D30" s="8" t="s">
+      <c r="E30" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="F30" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="E30" s="8" t="s">
+      <c r="G30" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="F30" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="G30" s="8" t="s">
+      <c r="H30" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="H30" s="8" t="s">
+      <c r="I30" s="8" t="s">
         <v>172</v>
-      </c>
-      <c r="I30" s="8" t="s">
-        <v>173</v>
       </c>
       <c r="J30" s="8" t="s">
         <v>19</v>
       </c>
       <c r="K30" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3027,10 +3006,10 @@
         <v>1</v>
       </c>
       <c r="C31" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>175</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>176</v>
       </c>
       <c r="E31" s="6" t="s">
         <v>176</v>
@@ -3042,19 +3021,19 @@
         <v>178</v>
       </c>
       <c r="H31" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I31" s="6" t="s">
         <v>179</v>
-      </c>
-      <c r="I31" s="6" t="s">
-        <v>180</v>
       </c>
       <c r="J31" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="n">
         <v>28</v>
       </c>
@@ -3062,34 +3041,34 @@
         <v>1</v>
       </c>
       <c r="C32" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="D32" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="D32" s="8" t="s">
+      <c r="E32" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="E32" s="8" t="s">
+      <c r="F32" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G32" s="8" t="s">
         <v>184</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="G32" s="8" t="s">
-        <v>186</v>
       </c>
       <c r="H32" s="8" t="s">
         <v>26</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="J32" s="8" t="s">
         <v>19</v>
       </c>
       <c r="K32" s="8" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="n">
         <v>29</v>
       </c>
@@ -3097,31 +3076,31 @@
         <v>1</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>33</v>
+        <v>177</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>192</v>
+        <v>178</v>
       </c>
       <c r="H33" s="6" t="s">
         <v>26</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="J33" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3132,31 +3111,31 @@
         <v>1</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="H34" s="8" t="s">
         <v>26</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="J34" s="8" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="K34" s="8" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3164,34 +3143,34 @@
         <v>31</v>
       </c>
       <c r="B35" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="H35" s="6" t="s">
         <v>26</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="J35" s="6" t="s">
         <v>28</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3199,37 +3178,37 @@
         <v>32</v>
       </c>
       <c r="B36" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>201</v>
+        <v>176</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>202</v>
+        <v>178</v>
       </c>
       <c r="H36" s="8" t="s">
         <v>26</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>203</v>
+        <v>179</v>
       </c>
       <c r="J36" s="8" t="s">
         <v>28</v>
       </c>
       <c r="K36" s="8" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="n">
         <v>33</v>
       </c>
@@ -3237,31 +3216,31 @@
         <v>2</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>26</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="J37" s="6" t="s">
         <v>28</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3272,31 +3251,31 @@
         <v>2</v>
       </c>
       <c r="C38" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="E38" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="D38" s="8" t="s">
+      <c r="F38" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="G38" s="8" t="s">
         <v>207</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="F38" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="G38" s="8" t="s">
-        <v>209</v>
       </c>
       <c r="H38" s="8" t="s">
         <v>26</v>
       </c>
       <c r="I38" s="8" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="J38" s="8" t="s">
         <v>28</v>
       </c>
       <c r="K38" s="8" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3307,104 +3286,104 @@
         <v>2</v>
       </c>
       <c r="C39" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="E39" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="F39" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="G39" s="6" t="s">
         <v>213</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="F39" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="G39" s="6" t="s">
-        <v>215</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>26</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="J39" s="6" t="s">
         <v>28</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="n">
         <v>36</v>
       </c>
       <c r="B40" s="7" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C40" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="E40" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="D40" s="8" t="s">
+      <c r="F40" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="G40" s="8" t="s">
         <v>219</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="F40" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="G40" s="8" t="s">
-        <v>221</v>
       </c>
       <c r="H40" s="8" t="s">
         <v>26</v>
       </c>
       <c r="I40" s="8" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="J40" s="8" t="s">
         <v>28</v>
       </c>
       <c r="K40" s="8" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="n">
         <v>37</v>
       </c>
       <c r="B41" s="5" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C41" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="E41" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="D41" s="6" t="s">
+      <c r="F41" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="G41" s="6" t="s">
         <v>225</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="G41" s="6" t="s">
-        <v>227</v>
       </c>
       <c r="H41" s="6" t="s">
         <v>26</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="K41" s="6" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="n">
         <v>38</v>
       </c>
@@ -3412,31 +3391,31 @@
         <v>1</v>
       </c>
       <c r="C42" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="E42" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="D42" s="8" t="s">
+      <c r="F42" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="G42" s="8" t="s">
         <v>231</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>232</v>
-      </c>
-      <c r="F42" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="G42" s="8" t="s">
-        <v>233</v>
       </c>
       <c r="H42" s="8" t="s">
         <v>26</v>
       </c>
       <c r="I42" s="8" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="J42" s="8" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="K42" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3447,31 +3426,31 @@
         <v>1</v>
       </c>
       <c r="C43" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="E43" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="F43" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="G43" s="6" t="s">
         <v>237</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="G43" s="6" t="s">
-        <v>239</v>
       </c>
       <c r="H43" s="6" t="s">
         <v>26</v>
       </c>
       <c r="I43" s="6" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="J43" s="6" t="s">
         <v>28</v>
       </c>
       <c r="K43" s="6" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3482,31 +3461,31 @@
         <v>1</v>
       </c>
       <c r="C44" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="E44" s="8" t="s">
         <v>242</v>
       </c>
-      <c r="D44" s="8" t="s">
+      <c r="F44" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="G44" s="8" t="s">
         <v>243</v>
-      </c>
-      <c r="E44" s="8" t="s">
-        <v>244</v>
-      </c>
-      <c r="F44" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="G44" s="8" t="s">
-        <v>245</v>
       </c>
       <c r="H44" s="8" t="s">
         <v>26</v>
       </c>
       <c r="I44" s="8" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="J44" s="8" t="s">
         <v>28</v>
       </c>
       <c r="K44" s="8" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3517,31 +3496,31 @@
         <v>1</v>
       </c>
       <c r="C45" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="E45" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="F45" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="G45" s="6" t="s">
         <v>249</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="F45" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="G45" s="6" t="s">
-        <v>251</v>
       </c>
       <c r="H45" s="6" t="s">
         <v>26</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="J45" s="6" t="s">
         <v>28</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3552,31 +3531,31 @@
         <v>1</v>
       </c>
       <c r="C46" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="E46" s="8" t="s">
         <v>254</v>
       </c>
-      <c r="D46" s="8" t="s">
+      <c r="F46" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="G46" s="8" t="s">
         <v>255</v>
-      </c>
-      <c r="E46" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="F46" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="G46" s="8" t="s">
-        <v>257</v>
       </c>
       <c r="H46" s="8" t="s">
         <v>26</v>
       </c>
       <c r="I46" s="8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="J46" s="8" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="K46" s="8" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3587,34 +3566,34 @@
         <v>1</v>
       </c>
       <c r="C47" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="E47" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="D47" s="6" t="s">
+      <c r="F47" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="G47" s="6" t="s">
         <v>261</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>262</v>
-      </c>
-      <c r="F47" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="G47" s="6" t="s">
-        <v>263</v>
       </c>
       <c r="H47" s="6" t="s">
         <v>26</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="J47" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="n">
         <v>44</v>
       </c>
@@ -3622,31 +3601,31 @@
         <v>1</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>267</v>
+        <v>223</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>268</v>
+        <v>224</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>269</v>
+        <v>225</v>
       </c>
       <c r="H48" s="8" t="s">
         <v>26</v>
       </c>
       <c r="I48" s="8" t="s">
-        <v>270</v>
+        <v>226</v>
       </c>
       <c r="J48" s="8" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="K48" s="8" t="s">
-        <v>271</v>
+        <v>227</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3657,31 +3636,31 @@
         <v>1</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="J49" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3692,31 +3671,31 @@
         <v>1</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="F50" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="G50" s="8" t="s">
         <v>275</v>
       </c>
-      <c r="G50" s="8" t="s">
-        <v>282</v>
-      </c>
       <c r="H50" s="8" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="I50" s="8" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="J50" s="8" t="s">
         <v>19</v>
       </c>
       <c r="K50" s="8" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3727,31 +3706,31 @@
         <v>1</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="J51" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3762,31 +3741,31 @@
         <v>1</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="H52" s="8" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="I52" s="8" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="J52" s="8" t="s">
         <v>19</v>
       </c>
       <c r="K52" s="8" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3797,31 +3776,31 @@
         <v>1</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="J53" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K53" s="6" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3832,31 +3811,31 @@
         <v>1</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="G54" s="8" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="H54" s="8" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I54" s="8" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="J54" s="8" t="s">
         <v>19</v>
       </c>
       <c r="K54" s="8" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3867,31 +3846,31 @@
         <v>1</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="J55" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K55" s="6" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3902,31 +3881,31 @@
         <v>1</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="F56" s="8" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="H56" s="8" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="I56" s="8" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="J56" s="8" t="s">
         <v>28</v>
       </c>
       <c r="K56" s="8" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3937,31 +3916,31 @@
         <v>1</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="G57" s="6" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="J57" s="6" t="s">
         <v>28</v>
       </c>
       <c r="K57" s="6" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3972,31 +3951,31 @@
         <v>1</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="F58" s="8" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="G58" s="8" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="H58" s="8" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="I58" s="8" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="J58" s="8" t="s">
         <v>19</v>
       </c>
       <c r="K58" s="8" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4007,31 +3986,31 @@
         <v>1</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="I59" s="6" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="J59" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K59" s="6" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4049,39 +4028,39 @@
     </row>
     <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="9" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="B61" s="10" t="n">
         <f aca="false">SUM(B5:B59)</f>
         <v>93</v>
       </c>
       <c r="C61" s="9" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="E61" s="11" t="n">
         <f aca="false">COUNTA(E5:E59)</f>
         <v>55</v>
       </c>
       <c r="F61" s="9" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="I61" s="9" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="J61" s="9" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="K61" s="9" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4099,7 +4078,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="12" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="12"/>
@@ -4149,142 +4128,142 @@
     </row>
     <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="B65" s="5" t="n">
         <v>8</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="G65" s="6" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="J65" s="6" t="s">
         <v>28</v>
       </c>
       <c r="K65" s="6" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="B66" s="5" t="n">
         <v>2</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="F66" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="G66" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="H66" s="6" t="s">
         <v>356</v>
       </c>
-      <c r="G66" s="6" t="s">
-        <v>356</v>
-      </c>
-      <c r="H66" s="6" t="s">
-        <v>363</v>
-      </c>
       <c r="I66" s="6" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="J66" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K66" s="6" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="B67" s="5" t="n">
         <v>4</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>367</v>
+        <v>360</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="G67" s="6" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="I67" s="6" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
       <c r="J67" s="6" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="K67" s="6" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
       <c r="B68" s="5" t="n">
         <v>1</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>376</v>
+        <v>369</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="H68" s="6" t="s">
         <v>26</v>
       </c>
       <c r="I68" s="6" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
       <c r="J68" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K68" s="6" t="s">
-        <v>379</v>
+        <v>372</v>
       </c>
     </row>
   </sheetData>
@@ -4310,7 +4289,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -4325,7 +4304,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>380</v>
+        <v>373</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4340,7 +4319,7 @@
     </row>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4356,7 +4335,7 @@
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3"/>
       <c r="B3" s="9" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="C3" s="14" t="n">
         <v>0.92</v>
@@ -4391,28 +4370,28 @@
         <v>4</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>383</v>
+        <v>376</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>384</v>
+        <v>377</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>386</v>
+        <v>379</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>387</v>
+        <v>380</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>388</v>
+        <v>381</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>389</v>
+        <v>382</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>12</v>
@@ -4432,7 +4411,7 @@
         <v>14</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
       <c r="F6" s="15" t="n">
         <v>0.69</v>
@@ -4449,10 +4428,10 @@
         <v>0.65</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>392</v>
+        <v>385</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4469,7 +4448,7 @@
         <v>23</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="F7" s="17" t="n">
         <v>0.0049</v>
@@ -4486,10 +4465,10 @@
         <v>0.0882</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>394</v>
+        <v>387</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4506,7 +4485,7 @@
         <v>32</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>395</v>
+        <v>388</v>
       </c>
       <c r="F8" s="15" t="n">
         <v>0.03</v>
@@ -4523,10 +4502,10 @@
         <v>0.05</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4543,7 +4522,7 @@
         <v>40</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>397</v>
+        <v>390</v>
       </c>
       <c r="F9" s="17" t="n">
         <v>0.1319</v>
@@ -4560,10 +4539,10 @@
         <v>0.0968</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4571,7 +4550,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>398</v>
+        <v>391</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>2</v>
@@ -4580,7 +4559,7 @@
         <v>46</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
       <c r="F10" s="15" t="n">
         <v>0.0205</v>
@@ -4597,10 +4576,10 @@
         <v>0.0318</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K10" s="8" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4608,7 +4587,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="C11" s="5" t="n">
         <v>3</v>
@@ -4617,7 +4596,7 @@
         <v>53</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
       <c r="F11" s="17" t="n">
         <v>0.0068</v>
@@ -4634,10 +4613,10 @@
         <v>0.0204</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>394</v>
+        <v>387</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4654,7 +4633,7 @@
         <v>60</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="F12" s="15" t="n">
         <v>0.0054</v>
@@ -4671,10 +4650,10 @@
         <v>0.0054</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4691,7 +4670,7 @@
         <v>66</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>403</v>
+        <v>396</v>
       </c>
       <c r="F13" s="17" t="n">
         <v>0.0287</v>
@@ -4708,10 +4687,10 @@
         <v>0.0287</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4728,7 +4707,7 @@
         <v>73</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0.0032</v>
@@ -4745,10 +4724,10 @@
         <v>0.0032</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4765,7 +4744,7 @@
         <v>78</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="F15" s="17" t="n">
         <v>0.0168</v>
@@ -4782,10 +4761,10 @@
         <v>0.0168</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>406</v>
+        <v>399</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4802,7 +4781,7 @@
         <v>84</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0.004</v>
@@ -4819,10 +4798,10 @@
         <v>0.004</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4839,7 +4818,7 @@
         <v>90</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="F17" s="17" t="n">
         <v>0.1953</v>
@@ -4856,10 +4835,10 @@
         <v>0.1953</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4876,7 +4855,7 @@
         <v>97</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>410</v>
+        <v>403</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0.002</v>
@@ -4893,13 +4872,13 @@
         <v>0.002</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="n">
         <v>14</v>
       </c>
@@ -4913,27 +4892,27 @@
         <v>102</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="F19" s="17" t="n">
-        <v>0.1</v>
+        <v>0.0657</v>
       </c>
       <c r="G19" s="18" t="n">
         <f aca="false">C19*F19</f>
-        <v>0.4</v>
+        <v>0.2628</v>
       </c>
       <c r="H19" s="17" t="n">
-        <v>0.08</v>
+        <v>0.055</v>
       </c>
       <c r="I19" s="18" t="n">
         <f aca="false">C19*H19</f>
-        <v>0.32</v>
+        <v>0.22</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>413</v>
+        <v>406</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4950,7 +4929,7 @@
         <v>110</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>414</v>
+        <v>407</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0.1082</v>
@@ -4967,10 +4946,10 @@
         <v>0.0851</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4987,27 +4966,27 @@
         <v>118</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>415</v>
+        <v>408</v>
       </c>
       <c r="F21" s="17" t="n">
-        <v>0.03</v>
+        <v>0.1729</v>
       </c>
       <c r="G21" s="18" t="n">
         <f aca="false">C21*F21</f>
-        <v>0.03</v>
+        <v>0.1729</v>
       </c>
       <c r="H21" s="17" t="n">
-        <v>0.02</v>
+        <v>0.1365</v>
       </c>
       <c r="I21" s="18" t="n">
         <f aca="false">C21*H21</f>
-        <v>0.02</v>
+        <v>0.1365</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>348</v>
+        <v>409</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5015,36 +4994,36 @@
         <v>17</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>124</v>
+        <v>410</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" s="8" t="s">
         <v>126</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="F22" s="15" t="n">
-        <v>0.1729</v>
+        <v>0.35</v>
       </c>
       <c r="G22" s="16" t="n">
         <f aca="false">C22*F22</f>
-        <v>0.1729</v>
+        <v>0.7</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>0.1365</v>
+        <v>0.25</v>
       </c>
       <c r="I22" s="16" t="n">
         <f aca="false">C22*H22</f>
-        <v>0.1365</v>
+        <v>0.5</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="K22" s="8" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5052,36 +5031,36 @@
         <v>18</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>134</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="F23" s="17" t="n">
-        <v>0.35</v>
+        <v>0.25</v>
       </c>
       <c r="G23" s="18" t="n">
         <f aca="false">C23*F23</f>
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="H23" s="17" t="n">
-        <v>0.25</v>
+        <v>0.18</v>
       </c>
       <c r="I23" s="18" t="n">
         <f aca="false">C23*H23</f>
-        <v>0.5</v>
+        <v>0.54</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5089,36 +5068,36 @@
         <v>19</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>421</v>
+        <v>145</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>0.25</v>
+        <v>0.0467</v>
       </c>
       <c r="G24" s="16" t="n">
         <f aca="false">C24*F24</f>
-        <v>0.75</v>
+        <v>0.0467</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>0.18</v>
+        <v>0.0388</v>
       </c>
       <c r="I24" s="16" t="n">
         <f aca="false">C24*H24</f>
-        <v>0.54</v>
+        <v>0.0388</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="K24" s="8" t="s">
-        <v>423</v>
+        <v>341</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5135,27 +5114,27 @@
         <v>155</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>424</v>
+        <v>417</v>
       </c>
       <c r="F25" s="17" t="n">
-        <v>0.0467</v>
+        <v>0.0185</v>
       </c>
       <c r="G25" s="18" t="n">
         <f aca="false">C25*F25</f>
-        <v>0.0467</v>
+        <v>0.0185</v>
       </c>
       <c r="H25" s="17" t="n">
-        <v>0.0388</v>
+        <v>0.0185</v>
       </c>
       <c r="I25" s="18" t="n">
         <f aca="false">C25*H25</f>
-        <v>0.0388</v>
+        <v>0.0185</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>348</v>
+        <v>418</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5163,36 +5142,36 @@
         <v>21</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C26" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>0.0185</v>
+        <v>0.12</v>
       </c>
       <c r="G26" s="16" t="n">
         <f aca="false">C26*F26</f>
-        <v>0.0185</v>
+        <v>0.12</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>0.0185</v>
+        <v>0.09</v>
       </c>
       <c r="I26" s="16" t="n">
         <f aca="false">C26*H26</f>
-        <v>0.0185</v>
+        <v>0.09</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="K26" s="8" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5200,36 +5179,36 @@
         <v>22</v>
       </c>
       <c r="B27" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="C27" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>170</v>
-      </c>
       <c r="E27" s="6" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="F27" s="17" t="n">
-        <v>0.12</v>
+        <v>0.1028</v>
       </c>
       <c r="G27" s="18" t="n">
         <f aca="false">C27*F27</f>
-        <v>0.12</v>
+        <v>0.1028</v>
       </c>
       <c r="H27" s="17" t="n">
-        <v>0.09</v>
+        <v>0.0831</v>
       </c>
       <c r="I27" s="18" t="n">
         <f aca="false">C27*H27</f>
-        <v>0.09</v>
+        <v>0.0831</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>428</v>
+        <v>409</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5237,36 +5216,36 @@
         <v>23</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>175</v>
+        <v>422</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D28" s="8" t="s">
         <v>176</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>0.1028</v>
+        <v>0.002</v>
       </c>
       <c r="G28" s="16" t="n">
         <f aca="false">C28*F28</f>
-        <v>0.1028</v>
+        <v>0.01</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>0.0831</v>
+        <v>0.002</v>
       </c>
       <c r="I28" s="16" t="n">
         <f aca="false">C28*H28</f>
-        <v>0.0831</v>
+        <v>0.01</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>417</v>
+        <v>341</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5274,36 +5253,36 @@
         <v>24</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>430</v>
+        <v>181</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>431</v>
+        <v>424</v>
       </c>
       <c r="F29" s="17" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G29" s="18" t="n">
         <f aca="false">C29*F29</f>
-        <v>0.01</v>
+        <v>0.003</v>
       </c>
       <c r="H29" s="17" t="n">
         <v>0.002</v>
       </c>
       <c r="I29" s="18" t="n">
         <f aca="false">C29*H29</f>
-        <v>0.01</v>
+        <v>0.002</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5311,36 +5290,36 @@
         <v>25</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>432</v>
+        <v>425</v>
       </c>
       <c r="F30" s="15" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G30" s="16" t="n">
         <f aca="false">C30*F30</f>
-        <v>0.003</v>
+        <v>0.008</v>
       </c>
       <c r="H30" s="15" t="n">
         <v>0.002</v>
       </c>
       <c r="I30" s="16" t="n">
         <f aca="false">C30*H30</f>
-        <v>0.002</v>
+        <v>0.008</v>
       </c>
       <c r="J30" s="8" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K30" s="8" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5348,36 +5327,36 @@
         <v>26</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>433</v>
+        <v>426</v>
       </c>
       <c r="F31" s="17" t="n">
         <v>0.002</v>
       </c>
       <c r="G31" s="18" t="n">
         <f aca="false">C31*F31</f>
-        <v>0.008</v>
+        <v>0.004</v>
       </c>
       <c r="H31" s="17" t="n">
         <v>0.002</v>
       </c>
       <c r="I31" s="18" t="n">
         <f aca="false">C31*H31</f>
-        <v>0.008</v>
+        <v>0.004</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5385,16 +5364,16 @@
         <v>27</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C32" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>434</v>
+        <v>427</v>
       </c>
       <c r="F32" s="15" t="n">
         <v>0.002</v>
@@ -5411,10 +5390,10 @@
         <v>0.004</v>
       </c>
       <c r="J32" s="8" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K32" s="8" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5422,16 +5401,16 @@
         <v>28</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>2</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>435</v>
+        <v>428</v>
       </c>
       <c r="F33" s="17" t="n">
         <v>0.002</v>
@@ -5448,84 +5427,84 @@
         <v>0.004</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="n">
         <v>29</v>
       </c>
       <c r="B34" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="D34" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="C34" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>220</v>
-      </c>
       <c r="E34" s="8" t="s">
-        <v>436</v>
+        <v>429</v>
       </c>
       <c r="F34" s="15" t="n">
         <v>0.002</v>
       </c>
       <c r="G34" s="16" t="n">
         <f aca="false">C34*F34</f>
-        <v>0.004</v>
+        <v>0.018</v>
       </c>
       <c r="H34" s="15" t="n">
         <v>0.002</v>
       </c>
       <c r="I34" s="16" t="n">
         <f aca="false">C34*H34</f>
-        <v>0.004</v>
+        <v>0.018</v>
       </c>
       <c r="J34" s="8" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K34" s="8" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="n">
         <v>30</v>
       </c>
       <c r="B35" s="6" t="s">
+        <v>430</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="C35" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>226</v>
-      </c>
       <c r="E35" s="6" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
       <c r="F35" s="17" t="n">
         <v>0.002</v>
       </c>
       <c r="G35" s="18" t="n">
         <f aca="false">C35*F35</f>
-        <v>0.018</v>
+        <v>0.004</v>
       </c>
       <c r="H35" s="17" t="n">
         <v>0.002</v>
       </c>
       <c r="I35" s="18" t="n">
         <f aca="false">C35*H35</f>
-        <v>0.018</v>
+        <v>0.004</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5533,16 +5512,16 @@
         <v>31</v>
       </c>
       <c r="B36" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="C36" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>232</v>
-      </c>
       <c r="E36" s="8" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="F36" s="15" t="n">
         <v>0.002</v>
@@ -5559,10 +5538,10 @@
         <v>0.002</v>
       </c>
       <c r="J36" s="8" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K36" s="8" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5570,16 +5549,16 @@
         <v>32</v>
       </c>
       <c r="B37" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="C37" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>238</v>
-      </c>
       <c r="E37" s="6" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
       <c r="F37" s="17" t="n">
         <v>0.002</v>
@@ -5596,10 +5575,10 @@
         <v>0.002</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5607,16 +5586,16 @@
         <v>33</v>
       </c>
       <c r="B38" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="8" t="s">
         <v>242</v>
       </c>
-      <c r="C38" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>244</v>
-      </c>
       <c r="E38" s="8" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
       <c r="F38" s="15" t="n">
         <v>0.002</v>
@@ -5633,10 +5612,10 @@
         <v>0.002</v>
       </c>
       <c r="J38" s="8" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K38" s="8" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5644,16 +5623,16 @@
         <v>34</v>
       </c>
       <c r="B39" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="C39" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>250</v>
-      </c>
       <c r="E39" s="6" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
       <c r="F39" s="17" t="n">
         <v>0.002</v>
@@ -5670,10 +5649,10 @@
         <v>0.002</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5681,16 +5660,16 @@
         <v>35</v>
       </c>
       <c r="B40" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="8" t="s">
         <v>254</v>
       </c>
-      <c r="C40" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>256</v>
-      </c>
       <c r="E40" s="8" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="F40" s="15" t="n">
         <v>0.002</v>
@@ -5707,10 +5686,10 @@
         <v>0.002</v>
       </c>
       <c r="J40" s="8" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K40" s="8" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5718,16 +5697,16 @@
         <v>36</v>
       </c>
       <c r="B41" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="C41" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>262</v>
-      </c>
       <c r="E41" s="6" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
       <c r="F41" s="17" t="n">
         <v>0.002</v>
@@ -5744,10 +5723,10 @@
         <v>0.002</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K41" s="6" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5755,44 +5734,44 @@
         <v>37</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C42" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="F42" s="15" t="n">
-        <v>0.002</v>
+        <v>3.0014</v>
       </c>
       <c r="G42" s="16" t="n">
         <f aca="false">C42*F42</f>
-        <v>0.002</v>
+        <v>3.0014</v>
       </c>
       <c r="H42" s="15" t="n">
-        <v>0.002</v>
+        <v>2.4748</v>
       </c>
       <c r="I42" s="16" t="n">
         <f aca="false">C42*H42</f>
-        <v>0.002</v>
+        <v>2.4748</v>
       </c>
       <c r="J42" s="8" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="K42" s="8" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="n">
         <v>38</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C43" s="5" t="n">
         <v>1</v>
@@ -5801,35 +5780,35 @@
         <v>274</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
       <c r="F43" s="17" t="n">
-        <v>3.0014</v>
+        <v>7.8102</v>
       </c>
       <c r="G43" s="18" t="n">
         <f aca="false">C43*F43</f>
-        <v>3.0014</v>
+        <v>7.8102</v>
       </c>
       <c r="H43" s="17" t="n">
-        <v>2.4748</v>
+        <v>5.8543</v>
       </c>
       <c r="I43" s="18" t="n">
         <f aca="false">C43*H43</f>
-        <v>2.4748</v>
+        <v>5.8543</v>
       </c>
       <c r="J43" s="6" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K43" s="6" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="n">
         <v>39</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C44" s="7" t="n">
         <v>1</v>
@@ -5838,30 +5817,30 @@
         <v>281</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
       <c r="F44" s="15" t="n">
-        <v>7.8102</v>
+        <v>3.6906</v>
       </c>
       <c r="G44" s="16" t="n">
         <f aca="false">C44*F44</f>
-        <v>7.8102</v>
+        <v>3.6906</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>5.8543</v>
+        <v>2.981</v>
       </c>
       <c r="I44" s="16" t="n">
         <f aca="false">C44*H44</f>
-        <v>5.8543</v>
+        <v>2.981</v>
       </c>
       <c r="J44" s="8" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K44" s="8" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="n">
         <v>40</v>
       </c>
@@ -5875,30 +5854,30 @@
         <v>288</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="F45" s="17" t="n">
-        <v>3.6906</v>
+        <v>3.9895</v>
       </c>
       <c r="G45" s="18" t="n">
         <f aca="false">C45*F45</f>
-        <v>3.6906</v>
+        <v>3.9895</v>
       </c>
       <c r="H45" s="17" t="n">
-        <v>2.981</v>
+        <v>3.9895</v>
       </c>
       <c r="I45" s="18" t="n">
         <f aca="false">C45*H45</f>
-        <v>2.981</v>
+        <v>3.9895</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="n">
         <v>41</v>
       </c>
@@ -5909,30 +5888,30 @@
         <v>1</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="F46" s="15" t="n">
-        <v>3.9895</v>
+        <v>0.6</v>
       </c>
       <c r="G46" s="16" t="n">
         <f aca="false">C46*F46</f>
-        <v>3.9895</v>
+        <v>0.6</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>3.9895</v>
+        <v>0.48</v>
       </c>
       <c r="I46" s="16" t="n">
         <f aca="false">C46*H46</f>
-        <v>3.9895</v>
+        <v>0.48</v>
       </c>
       <c r="J46" s="8" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="K46" s="8" t="s">
-        <v>450</v>
+        <v>341</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5940,36 +5919,36 @@
         <v>42</v>
       </c>
       <c r="B47" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="6" t="s">
         <v>300</v>
       </c>
-      <c r="C47" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>301</v>
-      </c>
       <c r="E47" s="6" t="s">
-        <v>451</v>
+        <v>445</v>
       </c>
       <c r="F47" s="17" t="n">
-        <v>0.6</v>
+        <v>0.1786</v>
       </c>
       <c r="G47" s="18" t="n">
         <f aca="false">C47*F47</f>
-        <v>0.6</v>
+        <v>0.1786</v>
       </c>
       <c r="H47" s="17" t="n">
-        <v>0.48</v>
+        <v>0.1375</v>
       </c>
       <c r="I47" s="18" t="n">
         <f aca="false">C47*H47</f>
-        <v>0.48</v>
+        <v>0.1375</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>348</v>
+        <v>409</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5977,36 +5956,36 @@
         <v>43</v>
       </c>
       <c r="B48" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="8" t="s">
         <v>306</v>
       </c>
-      <c r="C48" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>307</v>
-      </c>
       <c r="E48" s="8" t="s">
-        <v>452</v>
+        <v>446</v>
       </c>
       <c r="F48" s="15" t="n">
-        <v>0.1786</v>
+        <v>0.368</v>
       </c>
       <c r="G48" s="16" t="n">
         <f aca="false">C48*F48</f>
-        <v>0.1786</v>
+        <v>0.368</v>
       </c>
       <c r="H48" s="15" t="n">
-        <v>0.1375</v>
+        <v>0.2711</v>
       </c>
       <c r="I48" s="16" t="n">
         <f aca="false">C48*H48</f>
-        <v>0.1375</v>
+        <v>0.2711</v>
       </c>
       <c r="J48" s="8" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K48" s="8" t="s">
-        <v>417</v>
+        <v>341</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6014,7 +5993,7 @@
         <v>44</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C49" s="5" t="n">
         <v>1</v>
@@ -6023,27 +6002,27 @@
         <v>313</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="F49" s="17" t="n">
-        <v>0.368</v>
+        <v>1.6</v>
       </c>
       <c r="G49" s="18" t="n">
         <f aca="false">C49*F49</f>
-        <v>0.368</v>
+        <v>1.6</v>
       </c>
       <c r="H49" s="17" t="n">
-        <v>0.2711</v>
+        <v>1.3</v>
       </c>
       <c r="I49" s="18" t="n">
         <f aca="false">C49*H49</f>
-        <v>0.2711</v>
+        <v>1.3</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>348</v>
+        <v>448</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6051,7 +6030,7 @@
         <v>45</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C50" s="7" t="n">
         <v>1</v>
@@ -6060,27 +6039,27 @@
         <v>320</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
       <c r="F50" s="15" t="n">
-        <v>1.6</v>
+        <v>0.4186</v>
       </c>
       <c r="G50" s="16" t="n">
         <f aca="false">C50*F50</f>
-        <v>1.6</v>
+        <v>0.4186</v>
       </c>
       <c r="H50" s="15" t="n">
-        <v>1.3</v>
+        <v>0.3181</v>
       </c>
       <c r="I50" s="16" t="n">
         <f aca="false">C50*H50</f>
-        <v>1.3</v>
+        <v>0.3181</v>
       </c>
       <c r="J50" s="8" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="K50" s="8" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6088,39 +6067,39 @@
         <v>46</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C51" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
       <c r="F51" s="17" t="n">
-        <v>0.4186</v>
+        <v>3.6923</v>
       </c>
       <c r="G51" s="18" t="n">
         <f aca="false">C51*F51</f>
-        <v>0.4186</v>
+        <v>3.6923</v>
       </c>
       <c r="H51" s="17" t="n">
-        <v>0.3181</v>
+        <v>3.3626</v>
       </c>
       <c r="I51" s="18" t="n">
         <f aca="false">C51*H51</f>
-        <v>0.3181</v>
+        <v>3.3626</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="n">
         <v>47</v>
       </c>
@@ -6131,212 +6110,175 @@
         <v>1</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="F52" s="15" t="n">
-        <v>3.6923</v>
+        <v>0.3534</v>
       </c>
       <c r="G52" s="16" t="n">
         <f aca="false">C52*F52</f>
-        <v>3.6923</v>
+        <v>0.3534</v>
       </c>
       <c r="H52" s="15" t="n">
-        <v>3.3626</v>
+        <v>0.3534</v>
       </c>
       <c r="I52" s="16" t="n">
         <f aca="false">C52*H52</f>
-        <v>3.3626</v>
+        <v>0.3534</v>
       </c>
       <c r="J52" s="8" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="K52" s="8" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="5" t="n">
-        <v>48</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="C53" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D53" s="6" t="s">
-        <v>340</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>460</v>
-      </c>
-      <c r="F53" s="17" t="n">
-        <v>0.3534</v>
-      </c>
-      <c r="G53" s="18" t="n">
-        <f aca="false">C53*F53</f>
-        <v>0.3534</v>
-      </c>
-      <c r="H53" s="17" t="n">
-        <v>0.3534</v>
-      </c>
-      <c r="I53" s="18" t="n">
-        <f aca="false">C53*H53</f>
-        <v>0.3534</v>
-      </c>
-      <c r="J53" s="6" t="s">
-        <v>391</v>
-      </c>
-      <c r="K53" s="6" t="s">
-        <v>461</v>
-      </c>
+        <v>454</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3"/>
+      <c r="B53" s="3"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="3"/>
+      <c r="E53" s="3"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="3"/>
+      <c r="I53" s="3"/>
+      <c r="J53" s="3"/>
+      <c r="K53" s="3"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="3"/>
-      <c r="B54" s="3"/>
-      <c r="C54" s="3"/>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
-      <c r="F54" s="3"/>
-      <c r="G54" s="3"/>
-      <c r="H54" s="3"/>
-      <c r="I54" s="3"/>
-      <c r="J54" s="3"/>
-      <c r="K54" s="3"/>
+      <c r="A54" s="19"/>
+      <c r="B54" s="20" t="s">
+        <v>455</v>
+      </c>
+      <c r="C54" s="21" t="n">
+        <f aca="false">SUM(C6:C52)</f>
+        <v>93</v>
+      </c>
+      <c r="D54" s="19" t="s">
+        <v>456</v>
+      </c>
+      <c r="E54" s="19"/>
+      <c r="F54" s="19"/>
+      <c r="G54" s="22" t="n">
+        <f aca="false">SUM(G6:G52)</f>
+        <v>29.3384</v>
+      </c>
+      <c r="H54" s="19"/>
+      <c r="I54" s="22" t="n">
+        <f aca="false">SUM(I6:I52)</f>
+        <v>24.4929</v>
+      </c>
+      <c r="J54" s="19"/>
+      <c r="K54" s="19" t="s">
+        <v>457</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="19"/>
-      <c r="B55" s="20" t="s">
-        <v>462</v>
-      </c>
-      <c r="C55" s="21" t="n">
-        <f aca="false">SUM(C6:C53)</f>
-        <v>93</v>
-      </c>
-      <c r="D55" s="19" t="s">
-        <v>463</v>
-      </c>
+      <c r="B55" s="19" t="s">
+        <v>458</v>
+      </c>
+      <c r="C55" s="21"/>
+      <c r="D55" s="19"/>
       <c r="E55" s="19"/>
       <c r="F55" s="19"/>
-      <c r="G55" s="22" t="n">
-        <f aca="false">SUM(G6:G53)</f>
-        <v>29.5036</v>
+      <c r="G55" s="23" t="n">
+        <f aca="false">G54*C3</f>
+        <v>26.991328</v>
       </c>
       <c r="H55" s="19"/>
-      <c r="I55" s="22" t="n">
-        <f aca="false">SUM(I6:I53)</f>
-        <v>24.6109</v>
+      <c r="I55" s="23" t="n">
+        <f aca="false">I54*C3</f>
+        <v>22.533468</v>
       </c>
       <c r="J55" s="19"/>
       <c r="K55" s="19" t="s">
-        <v>464</v>
+        <v>459</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="19"/>
       <c r="B56" s="19" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="C56" s="21"/>
       <c r="D56" s="19"/>
       <c r="E56" s="19"/>
       <c r="F56" s="19"/>
       <c r="G56" s="23" t="n">
-        <f aca="false">G55*C3</f>
-        <v>27.143312</v>
+        <f aca="false">G54*10</f>
+        <v>293.384</v>
       </c>
       <c r="H56" s="19"/>
       <c r="I56" s="23" t="n">
-        <f aca="false">I55*C3</f>
-        <v>22.642028</v>
+        <f aca="false">I54*100</f>
+        <v>2449.29</v>
       </c>
       <c r="J56" s="19"/>
       <c r="K56" s="19" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="19"/>
       <c r="B57" s="19" t="s">
-        <v>467</v>
+        <v>462</v>
       </c>
       <c r="C57" s="21"/>
       <c r="D57" s="19"/>
       <c r="E57" s="19"/>
       <c r="F57" s="19"/>
-      <c r="G57" s="23" t="n">
-        <f aca="false">G55*10</f>
-        <v>295.036</v>
+      <c r="G57" s="24" t="n">
+        <f aca="false">(G43+G42+G44+G45)/G54</f>
+        <v>0.630289995364437</v>
       </c>
       <c r="H57" s="19"/>
-      <c r="I57" s="23" t="n">
-        <f aca="false">I55*100</f>
-        <v>2461.09</v>
+      <c r="I57" s="24" t="n">
+        <f aca="false">(I43+I42+I44+I45)/I54</f>
+        <v>0.624654491709842</v>
       </c>
       <c r="J57" s="19"/>
       <c r="K57" s="19" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="19"/>
-      <c r="B58" s="19" t="s">
-        <v>469</v>
-      </c>
-      <c r="C58" s="21"/>
-      <c r="D58" s="19"/>
-      <c r="E58" s="19"/>
-      <c r="F58" s="19"/>
-      <c r="G58" s="24" t="n">
-        <f aca="false">(G44+G43+G45+G46)/G55</f>
-        <v>0.626760802071612</v>
-      </c>
-      <c r="H58" s="19"/>
-      <c r="I58" s="24" t="n">
-        <f aca="false">(I44+I43+I45+I46)/I55</f>
-        <v>0.621659508591722</v>
-      </c>
-      <c r="J58" s="19"/>
-      <c r="K58" s="19" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="3"/>
-      <c r="B59" s="3"/>
-      <c r="C59" s="3"/>
-      <c r="D59" s="3"/>
-      <c r="E59" s="3"/>
-      <c r="F59" s="3"/>
-      <c r="G59" s="3"/>
-      <c r="H59" s="3"/>
-      <c r="I59" s="3"/>
-      <c r="J59" s="3"/>
-      <c r="K59" s="3"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="2" t="s">
-        <v>471</v>
-      </c>
-      <c r="B60" s="2"/>
-      <c r="C60" s="2"/>
-      <c r="D60" s="2"/>
-      <c r="E60" s="2"/>
-      <c r="F60" s="2"/>
-      <c r="G60" s="2"/>
-      <c r="H60" s="2"/>
-      <c r="I60" s="2"/>
-      <c r="J60" s="2"/>
-      <c r="K60" s="2"/>
+        <v>463</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="3"/>
+      <c r="B58" s="3"/>
+      <c r="C58" s="3"/>
+      <c r="D58" s="3"/>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="H58" s="3"/>
+      <c r="I58" s="3"/>
+      <c r="J58" s="3"/>
+      <c r="K58" s="3"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+      <c r="H59" s="2"/>
+      <c r="I59" s="2"/>
+      <c r="J59" s="2"/>
+      <c r="K59" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A60:K60"/>
+    <mergeCell ref="A59:K59"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
FC rev A: LED data level shifter U13, LEDs on VSYS (R49 removed)
- U13 SN74LV1T34DCKR (TI, LCSC C78541, SC-70-5) single-supply buffer powered
  from VSYS: TTL-level input (VIH <= 2.0 V), push-pull output at VSYS, so the
  XL-2020RGBC-WS2812B data input (VIH = 0.7 x VDD) is met on battery and on
  USB alone. C50 100 nF decoupling; R39 33R between U13 and D1.
- R49 0R removed: VLED merged into VSYS (LED supply unchanged in geometry,
  EMI at the magnetometer unchanged).
- PCB: U13/C50/R39 on the bottom next to D1, RGB data rerouted; DRC 0
  violations, 0 unconnected.
- BoM/JLC BoM/CPL (U13 correction 270 deg), costing, schematic PDF, Gerber,
  STEP, views regenerated; README and pin map updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0189Xg6tRAL4bRZ656VQBtPX
</commit_message>
<xml_diff>
--- a/00 - Docs/00 - FC_Docs/ACwing_FC_A_BoM.xlsx
+++ b/00 - Docs/00 - FC_Docs/ACwing_FC_A_BoM.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="833" uniqueCount="471">
   <si>
     <t xml:space="preserve">ACwing FC rev A - assembly BoM (1 board)</t>
   </si>
@@ -89,7 +89,7 @@
     <t xml:space="preserve">Johanson global P/N of the legacy 2450AT18A100E (same part). Left board edge, in the copper keep-out; R34 = 0R, C36 not fitted</t>
   </si>
   <si>
-    <t xml:space="preserve">C1, C12, C14, C15, C16, C17, C19, C21, C23, C24, C25, C26, C28, C39, C40, C41, C42, C45</t>
+    <t xml:space="preserve">C1, C12, C14, C15, C16, C17, C19, C21, C23, C24, C25, C26, C28, C39, C40, C41, C42, C45, C50</t>
   </si>
   <si>
     <t xml:space="preserve">100nF</t>
@@ -347,7 +347,7 @@
     <t xml:space="preserve">LED, RGB addressable, integrated driver, 2.0 x 2.0 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">Status LEDs D1 rear, D2 left, D3 front, D4 right: one chain from PA7 (TIM17_CH1 + DMA); D3 / D4 supply pins face away from the magnetometer. VDD 3.5-5.5 V (replaces WS2812B-2020, out of stock)</t>
+    <t xml:space="preserve">Status LEDs D1 rear, D2 left, D3 front, D4 right: one chain from PA7 (TIM17_CH1 + DMA); D3 / D4 supply pins face away from the magnetometer. VDD 3.5-5.5 V, supplied from VSYS; data through the U13 buffer (replaces WS2812B-2020, out of stock)</t>
   </si>
   <si>
     <t xml:space="preserve">D9</t>
@@ -707,7 +707,7 @@
     <t xml:space="preserve">Resistor, 0 Ohm jumper, 1/16 W</t>
   </si>
   <si>
-    <t xml:space="preserve">R34: antenna tuning, series position (replace with L/C after tuning); R49: VSYS -&gt; VLED link (replaces the Schottky). JLC Basic part</t>
+    <t xml:space="preserve">R34: antenna tuning, series position (replace with L/C after tuning). JLC Basic part</t>
   </si>
   <si>
     <t xml:space="preserve">R39</t>
@@ -818,9 +818,6 @@
     <t xml:space="preserve">Buck feedback, bottom. JLC Basic part</t>
   </si>
   <si>
-    <t xml:space="preserve">R49</t>
-  </si>
-  <si>
     <t xml:space="preserve">U1</t>
   </si>
   <si>
@@ -1019,6 +1016,24 @@
     <t xml:space="preserve">1S-6S input buck: VREG = 4.1 V (about VBAT on 1S). 350 in stock at LCSC on 2026-10-18: check before ordering</t>
   </si>
   <si>
+    <t xml:space="preserve">U13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SN74LV1T34DCKR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C78541</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SC-70-5 (SOT-353)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single buffer, single supply 1.6-5.5 V, TTL-level inputs (VIH 2.0 V at 5 V), 5 V tolerant, SC-70-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED data level shifter: PA7 (3.1-3.3 V) -&gt; VSYS level for the LED chain; VCC = VSYS, C50 decoupling; bottom side. LED data level shifter; ~24k in stock at LCSC on 2026-10-27</t>
+  </si>
+  <si>
     <t xml:space="preserve">Y1</t>
   </si>
   <si>
@@ -1316,9 +1331,6 @@
     <t xml:space="preserve">LCSC C25076 (JLC Basic)</t>
   </si>
   <si>
-    <t xml:space="preserve">R34, R49</t>
-  </si>
-  <si>
     <t xml:space="preserve">LCSC C17168 (JLC Basic)</t>
   </si>
   <si>
@@ -1383,6 +1395,12 @@
   </si>
   <si>
     <t xml:space="preserve">350 in stock on 2026-10-18 (30+ tier used for 100 boards)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LCSC C78541</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TI, ~24.5k in stock on 2026-10-27 (LED data level shifter)</t>
   </si>
   <si>
     <t xml:space="preserve">LCSC C843260</t>
@@ -2128,7 +2146,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>21</v>
@@ -2613,7 +2631,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="n">
         <v>16</v>
       </c>
@@ -3348,7 +3366,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="n">
         <v>37</v>
       </c>
@@ -3593,7 +3611,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="n">
         <v>44</v>
       </c>
@@ -3604,31 +3622,31 @@
         <v>264</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>223</v>
+        <v>265</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>224</v>
+        <v>266</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>177</v>
+        <v>267</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>225</v>
+        <v>268</v>
       </c>
       <c r="H48" s="8" t="s">
-        <v>26</v>
+        <v>269</v>
       </c>
       <c r="I48" s="8" t="s">
-        <v>226</v>
+        <v>270</v>
       </c>
       <c r="J48" s="8" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="K48" s="8" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="n">
         <v>45</v>
       </c>
@@ -3636,34 +3654,34 @@
         <v>1</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="E49" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="F49" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="F49" s="6" t="s">
-        <v>268</v>
-      </c>
       <c r="G49" s="6" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="J49" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="n">
         <v>46</v>
       </c>
@@ -3671,34 +3689,34 @@
         <v>1</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="H50" s="8" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="I50" s="8" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="J50" s="8" t="s">
         <v>19</v>
       </c>
       <c r="K50" s="8" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="n">
         <v>47</v>
       </c>
@@ -3706,34 +3724,34 @@
         <v>1</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="J51" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="n">
         <v>48</v>
       </c>
@@ -3741,31 +3759,31 @@
         <v>1</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="H52" s="8" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="I52" s="8" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="J52" s="8" t="s">
         <v>19</v>
       </c>
       <c r="K52" s="8" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3776,34 +3794,34 @@
         <v>1</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="J53" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K53" s="6" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="n">
         <v>50</v>
       </c>
@@ -3811,31 +3829,31 @@
         <v>1</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G54" s="8" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="H54" s="8" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="I54" s="8" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="J54" s="8" t="s">
         <v>19</v>
       </c>
       <c r="K54" s="8" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3846,31 +3864,31 @@
         <v>1</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>268</v>
+        <v>313</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="J55" s="6" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="K55" s="6" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3881,31 +3899,31 @@
         <v>1</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="F56" s="8" t="s">
-        <v>314</v>
+        <v>267</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="H56" s="8" t="s">
-        <v>316</v>
+        <v>295</v>
       </c>
       <c r="I56" s="8" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="J56" s="8" t="s">
         <v>28</v>
       </c>
       <c r="K56" s="8" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3916,34 +3934,34 @@
         <v>1</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>268</v>
+        <v>325</v>
       </c>
       <c r="G57" s="6" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>296</v>
+        <v>327</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="J57" s="6" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="K57" s="6" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="n">
         <v>54</v>
       </c>
@@ -3951,31 +3969,31 @@
         <v>1</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D58" s="8" t="s">
+        <v>331</v>
+      </c>
+      <c r="E58" s="8" t="s">
+        <v>331</v>
+      </c>
+      <c r="F58" s="8" t="s">
         <v>325</v>
       </c>
-      <c r="E58" s="8" t="s">
-        <v>325</v>
-      </c>
-      <c r="F58" s="8" t="s">
-        <v>326</v>
-      </c>
       <c r="G58" s="8" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="H58" s="8" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="I58" s="8" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="J58" s="8" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="K58" s="8" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3986,31 +4004,31 @@
         <v>1</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="I59" s="6" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="J59" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K59" s="6" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4028,39 +4046,39 @@
     </row>
     <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="9" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="B61" s="10" t="n">
         <f aca="false">SUM(B5:B59)</f>
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C61" s="9" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="E61" s="11" t="n">
         <f aca="false">COUNTA(E5:E59)</f>
         <v>55</v>
       </c>
       <c r="F61" s="9" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="I61" s="9" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="J61" s="9" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="K61" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4078,7 +4096,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="12" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="12"/>
@@ -4128,142 +4146,142 @@
     </row>
     <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="B65" s="5" t="n">
         <v>8</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="G65" s="6" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="J65" s="6" t="s">
         <v>28</v>
       </c>
       <c r="K65" s="6" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B66" s="5" t="n">
         <v>2</v>
       </c>
       <c r="C66" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="E66" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="F66" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="D66" s="6" t="s">
-        <v>355</v>
-      </c>
-      <c r="E66" s="6" t="s">
-        <v>348</v>
-      </c>
-      <c r="F66" s="6" t="s">
-        <v>349</v>
-      </c>
       <c r="G66" s="6" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="I66" s="6" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="J66" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K66" s="6" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B67" s="5" t="n">
         <v>4</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="G67" s="6" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="I67" s="6" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="J67" s="6" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="K67" s="6" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="B68" s="5" t="n">
         <v>1</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="H68" s="6" t="s">
         <v>26</v>
       </c>
       <c r="I68" s="6" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="J68" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K68" s="6" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
     </row>
   </sheetData>
@@ -4289,7 +4307,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -4304,7 +4322,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4319,7 +4337,7 @@
     </row>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4335,7 +4353,7 @@
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3"/>
       <c r="B3" s="9" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="C3" s="14" t="n">
         <v>0.92</v>
@@ -4370,28 +4388,28 @@
         <v>4</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>12</v>
@@ -4411,7 +4429,7 @@
         <v>14</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="F6" s="15" t="n">
         <v>0.69</v>
@@ -4428,10 +4446,10 @@
         <v>0.65</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4442,33 +4460,33 @@
         <v>21</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>23</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="F7" s="17" t="n">
         <v>0.0049</v>
       </c>
       <c r="G7" s="18" t="n">
         <f aca="false">C7*F7</f>
-        <v>0.0882</v>
+        <v>0.0931</v>
       </c>
       <c r="H7" s="17" t="n">
         <v>0.0049</v>
       </c>
       <c r="I7" s="18" t="n">
         <f aca="false">C7*H7</f>
-        <v>0.0882</v>
+        <v>0.0931</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4485,7 +4503,7 @@
         <v>32</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="F8" s="15" t="n">
         <v>0.03</v>
@@ -4502,10 +4520,10 @@
         <v>0.05</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4522,7 +4540,7 @@
         <v>40</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="F9" s="17" t="n">
         <v>0.1319</v>
@@ -4539,10 +4557,10 @@
         <v>0.0968</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4550,7 +4568,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>2</v>
@@ -4559,7 +4577,7 @@
         <v>46</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="F10" s="15" t="n">
         <v>0.0205</v>
@@ -4576,10 +4594,10 @@
         <v>0.0318</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K10" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4587,7 +4605,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="C11" s="5" t="n">
         <v>3</v>
@@ -4596,7 +4614,7 @@
         <v>53</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="F11" s="17" t="n">
         <v>0.0068</v>
@@ -4613,10 +4631,10 @@
         <v>0.0204</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4633,7 +4651,7 @@
         <v>60</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="F12" s="15" t="n">
         <v>0.0054</v>
@@ -4650,10 +4668,10 @@
         <v>0.0054</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4670,7 +4688,7 @@
         <v>66</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="F13" s="17" t="n">
         <v>0.0287</v>
@@ -4687,10 +4705,10 @@
         <v>0.0287</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4707,7 +4725,7 @@
         <v>73</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0.0032</v>
@@ -4724,10 +4742,10 @@
         <v>0.0032</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4744,7 +4762,7 @@
         <v>78</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="F15" s="17" t="n">
         <v>0.0168</v>
@@ -4761,10 +4779,10 @@
         <v>0.0168</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4781,7 +4799,7 @@
         <v>84</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0.004</v>
@@ -4798,10 +4816,10 @@
         <v>0.004</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4818,7 +4836,7 @@
         <v>90</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="F17" s="17" t="n">
         <v>0.1953</v>
@@ -4835,10 +4853,10 @@
         <v>0.1953</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4855,7 +4873,7 @@
         <v>97</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0.002</v>
@@ -4872,10 +4890,10 @@
         <v>0.002</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4892,7 +4910,7 @@
         <v>102</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="F19" s="17" t="n">
         <v>0.0657</v>
@@ -4909,10 +4927,10 @@
         <v>0.22</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4929,7 +4947,7 @@
         <v>110</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0.1082</v>
@@ -4946,10 +4964,10 @@
         <v>0.0851</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4966,7 +4984,7 @@
         <v>118</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="F21" s="17" t="n">
         <v>0.1729</v>
@@ -4983,10 +5001,10 @@
         <v>0.1365</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4994,7 +5012,7 @@
         <v>17</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="C22" s="7" t="n">
         <v>2</v>
@@ -5003,7 +5021,7 @@
         <v>126</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0.35</v>
@@ -5020,10 +5038,10 @@
         <v>0.5</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K22" s="8" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5031,7 +5049,7 @@
         <v>18</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="C23" s="5" t="n">
         <v>3</v>
@@ -5040,7 +5058,7 @@
         <v>134</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="F23" s="17" t="n">
         <v>0.25</v>
@@ -5057,10 +5075,10 @@
         <v>0.54</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5077,7 +5095,7 @@
         <v>147</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0.0467</v>
@@ -5094,10 +5112,10 @@
         <v>0.0388</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K24" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5114,7 +5132,7 @@
         <v>155</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="F25" s="17" t="n">
         <v>0.0185</v>
@@ -5131,10 +5149,10 @@
         <v>0.0185</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5151,7 +5169,7 @@
         <v>162</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="F26" s="15" t="n">
         <v>0.12</v>
@@ -5168,10 +5186,10 @@
         <v>0.09</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K26" s="8" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5188,7 +5206,7 @@
         <v>168</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="F27" s="17" t="n">
         <v>0.1028</v>
@@ -5205,10 +5223,10 @@
         <v>0.0831</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5216,7 +5234,7 @@
         <v>23</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="C28" s="7" t="n">
         <v>5</v>
@@ -5225,7 +5243,7 @@
         <v>176</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
       <c r="F28" s="15" t="n">
         <v>0.002</v>
@@ -5242,10 +5260,10 @@
         <v>0.01</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5262,7 +5280,7 @@
         <v>183</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="F29" s="17" t="n">
         <v>0.003</v>
@@ -5279,10 +5297,10 @@
         <v>0.002</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5299,7 +5317,7 @@
         <v>193</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="F30" s="15" t="n">
         <v>0.002</v>
@@ -5316,10 +5334,10 @@
         <v>0.008</v>
       </c>
       <c r="J30" s="8" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K30" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5336,7 +5354,7 @@
         <v>200</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="F31" s="17" t="n">
         <v>0.002</v>
@@ -5353,10 +5371,10 @@
         <v>0.004</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5373,7 +5391,7 @@
         <v>206</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="F32" s="15" t="n">
         <v>0.002</v>
@@ -5390,10 +5408,10 @@
         <v>0.004</v>
       </c>
       <c r="J32" s="8" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K32" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5410,7 +5428,7 @@
         <v>212</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
       <c r="F33" s="17" t="n">
         <v>0.002</v>
@@ -5427,10 +5445,10 @@
         <v>0.004</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5447,7 +5465,7 @@
         <v>218</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="F34" s="15" t="n">
         <v>0.002</v>
@@ -5464,10 +5482,10 @@
         <v>0.018</v>
       </c>
       <c r="J34" s="8" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K34" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5475,36 +5493,36 @@
         <v>30</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>430</v>
+        <v>222</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>224</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="F35" s="17" t="n">
         <v>0.002</v>
       </c>
       <c r="G35" s="18" t="n">
         <f aca="false">C35*F35</f>
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="H35" s="17" t="n">
         <v>0.002</v>
       </c>
       <c r="I35" s="18" t="n">
         <f aca="false">C35*H35</f>
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5521,7 +5539,7 @@
         <v>230</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="F36" s="15" t="n">
         <v>0.002</v>
@@ -5538,10 +5556,10 @@
         <v>0.002</v>
       </c>
       <c r="J36" s="8" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K36" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5558,7 +5576,7 @@
         <v>236</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="F37" s="17" t="n">
         <v>0.002</v>
@@ -5575,10 +5593,10 @@
         <v>0.002</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5595,7 +5613,7 @@
         <v>242</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="F38" s="15" t="n">
         <v>0.002</v>
@@ -5612,10 +5630,10 @@
         <v>0.002</v>
       </c>
       <c r="J38" s="8" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K38" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5632,7 +5650,7 @@
         <v>248</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="F39" s="17" t="n">
         <v>0.002</v>
@@ -5649,10 +5667,10 @@
         <v>0.002</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5669,7 +5687,7 @@
         <v>254</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="F40" s="15" t="n">
         <v>0.002</v>
@@ -5686,10 +5704,10 @@
         <v>0.002</v>
       </c>
       <c r="J40" s="8" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K40" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5706,7 +5724,7 @@
         <v>260</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="F41" s="17" t="n">
         <v>0.002</v>
@@ -5723,10 +5741,10 @@
         <v>0.002</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K41" s="6" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5734,16 +5752,16 @@
         <v>37</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C42" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="F42" s="15" t="n">
         <v>3.0014</v>
@@ -5760,10 +5778,10 @@
         <v>2.4748</v>
       </c>
       <c r="J42" s="8" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K42" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5771,16 +5789,16 @@
         <v>38</v>
       </c>
       <c r="B43" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="C43" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>274</v>
-      </c>
       <c r="E43" s="6" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="F43" s="17" t="n">
         <v>7.8102</v>
@@ -5797,10 +5815,10 @@
         <v>5.8543</v>
       </c>
       <c r="J43" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K43" s="6" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5808,16 +5826,16 @@
         <v>39</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C44" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="F44" s="15" t="n">
         <v>3.6906</v>
@@ -5834,10 +5852,10 @@
         <v>2.981</v>
       </c>
       <c r="J44" s="8" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K44" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5845,16 +5863,16 @@
         <v>40</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C45" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="F45" s="17" t="n">
         <v>3.9895</v>
@@ -5871,10 +5889,10 @@
         <v>3.9895</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5882,16 +5900,16 @@
         <v>41</v>
       </c>
       <c r="B46" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="C46" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="C46" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>294</v>
-      </c>
       <c r="E46" s="8" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="F46" s="15" t="n">
         <v>0.6</v>
@@ -5908,10 +5926,10 @@
         <v>0.48</v>
       </c>
       <c r="J46" s="8" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K46" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5919,16 +5937,16 @@
         <v>42</v>
       </c>
       <c r="B47" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="6" t="s">
         <v>299</v>
       </c>
-      <c r="C47" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>300</v>
-      </c>
       <c r="E47" s="6" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="F47" s="17" t="n">
         <v>0.1786</v>
@@ -5945,10 +5963,10 @@
         <v>0.1375</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5956,16 +5974,16 @@
         <v>43</v>
       </c>
       <c r="B48" s="8" t="s">
+        <v>304</v>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="C48" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>306</v>
-      </c>
       <c r="E48" s="8" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="F48" s="15" t="n">
         <v>0.368</v>
@@ -5982,10 +6000,10 @@
         <v>0.2711</v>
       </c>
       <c r="J48" s="8" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K48" s="8" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5993,16 +6011,16 @@
         <v>44</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C49" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="F49" s="17" t="n">
         <v>1.6</v>
@@ -6019,10 +6037,10 @@
         <v>1.3</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6030,16 +6048,16 @@
         <v>45</v>
       </c>
       <c r="B50" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C50" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="8" t="s">
         <v>319</v>
       </c>
-      <c r="C50" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>320</v>
-      </c>
       <c r="E50" s="8" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="F50" s="15" t="n">
         <v>0.4186</v>
@@ -6056,10 +6074,10 @@
         <v>0.3181</v>
       </c>
       <c r="J50" s="8" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K50" s="8" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6067,16 +6085,16 @@
         <v>46</v>
       </c>
       <c r="B51" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="C51" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="C51" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" s="6" t="s">
-        <v>325</v>
-      </c>
       <c r="E51" s="6" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="F51" s="17" t="n">
         <v>3.6923</v>
@@ -6093,192 +6111,229 @@
         <v>3.3626</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="n">
         <v>47</v>
       </c>
       <c r="B52" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="C52" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="8" t="s">
         <v>331</v>
       </c>
-      <c r="C52" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D52" s="8" t="s">
-        <v>333</v>
-      </c>
       <c r="E52" s="8" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="F52" s="15" t="n">
-        <v>0.3534</v>
+        <v>0.0593</v>
       </c>
       <c r="G52" s="16" t="n">
         <f aca="false">C52*F52</f>
-        <v>0.3534</v>
+        <v>0.0593</v>
       </c>
       <c r="H52" s="15" t="n">
-        <v>0.3534</v>
+        <v>0.0593</v>
       </c>
       <c r="I52" s="16" t="n">
         <f aca="false">C52*H52</f>
+        <v>0.0593</v>
+      </c>
+      <c r="J52" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="K52" s="8" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="C53" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="F53" s="17" t="n">
         <v>0.3534</v>
       </c>
-      <c r="J52" s="8" t="s">
-        <v>384</v>
-      </c>
-      <c r="K52" s="8" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3"/>
-      <c r="B53" s="3"/>
-      <c r="C53" s="3"/>
-      <c r="D53" s="3"/>
-      <c r="E53" s="3"/>
-      <c r="F53" s="3"/>
-      <c r="G53" s="3"/>
-      <c r="H53" s="3"/>
-      <c r="I53" s="3"/>
-      <c r="J53" s="3"/>
-      <c r="K53" s="3"/>
+      <c r="G53" s="18" t="n">
+        <f aca="false">C53*F53</f>
+        <v>0.3534</v>
+      </c>
+      <c r="H53" s="17" t="n">
+        <v>0.3534</v>
+      </c>
+      <c r="I53" s="18" t="n">
+        <f aca="false">C53*H53</f>
+        <v>0.3534</v>
+      </c>
+      <c r="J53" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="K53" s="6" t="s">
+        <v>460</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="19"/>
-      <c r="B54" s="20" t="s">
-        <v>455</v>
-      </c>
-      <c r="C54" s="21" t="n">
-        <f aca="false">SUM(C6:C52)</f>
-        <v>93</v>
-      </c>
-      <c r="D54" s="19" t="s">
-        <v>456</v>
-      </c>
-      <c r="E54" s="19"/>
-      <c r="F54" s="19"/>
-      <c r="G54" s="22" t="n">
-        <f aca="false">SUM(G6:G52)</f>
-        <v>29.3384</v>
-      </c>
-      <c r="H54" s="19"/>
-      <c r="I54" s="22" t="n">
-        <f aca="false">SUM(I6:I52)</f>
-        <v>24.4929</v>
-      </c>
-      <c r="J54" s="19"/>
-      <c r="K54" s="19" t="s">
-        <v>457</v>
-      </c>
+      <c r="A54" s="3"/>
+      <c r="B54" s="3"/>
+      <c r="C54" s="3"/>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="3"/>
+      <c r="J54" s="3"/>
+      <c r="K54" s="3"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="19"/>
-      <c r="B55" s="19" t="s">
-        <v>458</v>
-      </c>
-      <c r="C55" s="21"/>
-      <c r="D55" s="19"/>
+      <c r="B55" s="20" t="s">
+        <v>461</v>
+      </c>
+      <c r="C55" s="21" t="n">
+        <f aca="false">SUM(C6:C53)</f>
+        <v>94</v>
+      </c>
+      <c r="D55" s="19" t="s">
+        <v>462</v>
+      </c>
       <c r="E55" s="19"/>
       <c r="F55" s="19"/>
-      <c r="G55" s="23" t="n">
-        <f aca="false">G54*C3</f>
-        <v>26.991328</v>
+      <c r="G55" s="22" t="n">
+        <f aca="false">SUM(G6:G53)</f>
+        <v>29.4006</v>
       </c>
       <c r="H55" s="19"/>
-      <c r="I55" s="23" t="n">
-        <f aca="false">I54*C3</f>
-        <v>22.533468</v>
+      <c r="I55" s="22" t="n">
+        <f aca="false">SUM(I6:I53)</f>
+        <v>24.5551</v>
       </c>
       <c r="J55" s="19"/>
       <c r="K55" s="19" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="19"/>
       <c r="B56" s="19" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="C56" s="21"/>
       <c r="D56" s="19"/>
       <c r="E56" s="19"/>
       <c r="F56" s="19"/>
       <c r="G56" s="23" t="n">
-        <f aca="false">G54*10</f>
-        <v>293.384</v>
+        <f aca="false">G55*C3</f>
+        <v>27.048552</v>
       </c>
       <c r="H56" s="19"/>
       <c r="I56" s="23" t="n">
-        <f aca="false">I54*100</f>
-        <v>2449.29</v>
+        <f aca="false">I55*C3</f>
+        <v>22.590692</v>
       </c>
       <c r="J56" s="19"/>
       <c r="K56" s="19" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="19"/>
       <c r="B57" s="19" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="C57" s="21"/>
       <c r="D57" s="19"/>
       <c r="E57" s="19"/>
       <c r="F57" s="19"/>
-      <c r="G57" s="24" t="n">
-        <f aca="false">(G43+G42+G44+G45)/G54</f>
-        <v>0.630289995364437</v>
+      <c r="G57" s="23" t="n">
+        <f aca="false">G55*10</f>
+        <v>294.006</v>
       </c>
       <c r="H57" s="19"/>
-      <c r="I57" s="24" t="n">
-        <f aca="false">(I43+I42+I44+I45)/I54</f>
-        <v>0.624654491709842</v>
+      <c r="I57" s="23" t="n">
+        <f aca="false">I55*100</f>
+        <v>2455.51</v>
       </c>
       <c r="J57" s="19"/>
       <c r="K57" s="19" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3"/>
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="3"/>
-      <c r="E58" s="3"/>
-      <c r="F58" s="3"/>
-      <c r="G58" s="3"/>
-      <c r="H58" s="3"/>
-      <c r="I58" s="3"/>
-      <c r="J58" s="3"/>
-      <c r="K58" s="3"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="2" t="s">
-        <v>464</v>
-      </c>
-      <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-      <c r="E59" s="2"/>
-      <c r="F59" s="2"/>
-      <c r="G59" s="2"/>
-      <c r="H59" s="2"/>
-      <c r="I59" s="2"/>
-      <c r="J59" s="2"/>
-      <c r="K59" s="2"/>
+        <v>467</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="19"/>
+      <c r="B58" s="19" t="s">
+        <v>468</v>
+      </c>
+      <c r="C58" s="21"/>
+      <c r="D58" s="19"/>
+      <c r="E58" s="19"/>
+      <c r="F58" s="19"/>
+      <c r="G58" s="24" t="n">
+        <f aca="false">(G43+G42+G44+G45)/G55</f>
+        <v>0.628956551907104</v>
+      </c>
+      <c r="H58" s="19"/>
+      <c r="I58" s="24" t="n">
+        <f aca="false">(I43+I42+I44+I45)/I55</f>
+        <v>0.623072192742037</v>
+      </c>
+      <c r="J58" s="19"/>
+      <c r="K58" s="19" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="3"/>
+      <c r="B59" s="3"/>
+      <c r="C59" s="3"/>
+      <c r="D59" s="3"/>
+      <c r="E59" s="3"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+      <c r="H59" s="3"/>
+      <c r="I59" s="3"/>
+      <c r="J59" s="3"/>
+      <c r="K59" s="3"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2"/>
+      <c r="F60" s="2"/>
+      <c r="G60" s="2"/>
+      <c r="H60" s="2"/>
+      <c r="I60" s="2"/>
+      <c r="J60" s="2"/>
+      <c r="K60" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A59:K59"/>
+    <mergeCell ref="A60:K60"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>